<commit_message>
Regrouping policy domain alcohol
changed:
- social and living environment in domain living environment
- control of production in domain other
</commit_message>
<xml_diff>
--- a/data/phi_raw_data.xlsx
+++ b/data/phi_raw_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carolinkilian/Desktop/Research projects/Public Health Index/Github/Public-Health-Index/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E3CA47-6DBE-7C40-BC12-766826A8D584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1064BCF0-0795-4F44-91E5-FCAAAF982F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{07406E1C-1769-574D-9B9C-B78BFD08E78B}"/>
   </bookViews>
@@ -246,9 +246,6 @@
     <t>active living environments</t>
   </si>
   <si>
-    <t>social and living environmental controls</t>
-  </si>
-  <si>
     <t>fctc</t>
   </si>
   <si>
@@ -259,6 +256,9 @@
   </si>
   <si>
     <t>Physical inactivity</t>
+  </si>
+  <si>
+    <t>social and environmental controls</t>
   </si>
 </sst>
 </file>
@@ -647,6 +647,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55F2ECBD-B66B-9E43-893D-B37A0B73B8F5}">
   <dimension ref="A1:G469"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="22.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -676,7 +679,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
         <v>65</v>
@@ -699,7 +702,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
         <v>65</v>
@@ -722,7 +725,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
         <v>65</v>
@@ -745,7 +748,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
         <v>65</v>
@@ -768,7 +771,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
         <v>65</v>
@@ -791,7 +794,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C7" t="s">
         <v>65</v>
@@ -814,7 +817,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
         <v>65</v>
@@ -837,7 +840,7 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
         <v>65</v>
@@ -860,7 +863,7 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
         <v>65</v>
@@ -883,7 +886,7 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
         <v>65</v>
@@ -906,7 +909,7 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
         <v>65</v>
@@ -929,7 +932,7 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C13" t="s">
         <v>65</v>
@@ -952,7 +955,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
         <v>65</v>
@@ -975,7 +978,7 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
         <v>65</v>
@@ -998,7 +1001,7 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
         <v>65</v>
@@ -1021,7 +1024,7 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
         <v>65</v>
@@ -1044,7 +1047,7 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
         <v>65</v>
@@ -1067,7 +1070,7 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
         <v>65</v>
@@ -1090,7 +1093,7 @@
         <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C20" t="s">
         <v>65</v>
@@ -1113,7 +1116,7 @@
         <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1136,7 +1139,7 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C22" t="s">
         <v>65</v>
@@ -1159,7 +1162,7 @@
         <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C23" t="s">
         <v>65</v>
@@ -1182,7 +1185,7 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C24" t="s">
         <v>65</v>
@@ -1205,7 +1208,7 @@
         <v>9</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C25" t="s">
         <v>65</v>
@@ -1228,7 +1231,7 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C26" t="s">
         <v>65</v>
@@ -1251,7 +1254,7 @@
         <v>11</v>
       </c>
       <c r="B27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C27" t="s">
         <v>65</v>
@@ -1274,7 +1277,7 @@
         <v>12</v>
       </c>
       <c r="B28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
         <v>65</v>
@@ -1297,7 +1300,7 @@
         <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
         <v>65</v>
@@ -1320,7 +1323,7 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C30" t="s">
         <v>65</v>
@@ -1343,7 +1346,7 @@
         <v>15</v>
       </c>
       <c r="B31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C31" t="s">
         <v>65</v>
@@ -1366,7 +1369,7 @@
         <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C32" t="s">
         <v>65</v>
@@ -1389,7 +1392,7 @@
         <v>17</v>
       </c>
       <c r="B33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C33" t="s">
         <v>65</v>
@@ -1412,7 +1415,7 @@
         <v>18</v>
       </c>
       <c r="B34" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C34" t="s">
         <v>65</v>
@@ -1435,7 +1438,7 @@
         <v>19</v>
       </c>
       <c r="B35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C35" t="s">
         <v>65</v>
@@ -1458,7 +1461,7 @@
         <v>20</v>
       </c>
       <c r="B36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C36" t="s">
         <v>65</v>
@@ -1481,7 +1484,7 @@
         <v>21</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C37" t="s">
         <v>65</v>
@@ -1504,10 +1507,10 @@
         <v>4</v>
       </c>
       <c r="B38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D38" t="s">
         <v>25</v>
@@ -1527,10 +1530,10 @@
         <v>5</v>
       </c>
       <c r="B39" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D39" t="s">
         <v>25</v>
@@ -1550,10 +1553,10 @@
         <v>6</v>
       </c>
       <c r="B40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D40" t="s">
         <v>25</v>
@@ -1573,10 +1576,10 @@
         <v>7</v>
       </c>
       <c r="B41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D41" t="s">
         <v>25</v>
@@ -1596,10 +1599,10 @@
         <v>8</v>
       </c>
       <c r="B42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C42" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D42" t="s">
         <v>25</v>
@@ -1619,10 +1622,10 @@
         <v>9</v>
       </c>
       <c r="B43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D43" t="s">
         <v>25</v>
@@ -1642,10 +1645,10 @@
         <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D44" t="s">
         <v>25</v>
@@ -1665,10 +1668,10 @@
         <v>11</v>
       </c>
       <c r="B45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D45" t="s">
         <v>25</v>
@@ -1688,10 +1691,10 @@
         <v>12</v>
       </c>
       <c r="B46" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C46" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D46" t="s">
         <v>25</v>
@@ -1711,10 +1714,10 @@
         <v>13</v>
       </c>
       <c r="B47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C47" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D47" t="s">
         <v>25</v>
@@ -1734,10 +1737,10 @@
         <v>14</v>
       </c>
       <c r="B48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C48" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D48" t="s">
         <v>25</v>
@@ -1757,10 +1760,10 @@
         <v>15</v>
       </c>
       <c r="B49" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C49" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D49" t="s">
         <v>25</v>
@@ -1780,10 +1783,10 @@
         <v>16</v>
       </c>
       <c r="B50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C50" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D50" t="s">
         <v>25</v>
@@ -1803,10 +1806,10 @@
         <v>17</v>
       </c>
       <c r="B51" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C51" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D51" t="s">
         <v>25</v>
@@ -1826,10 +1829,10 @@
         <v>18</v>
       </c>
       <c r="B52" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C52" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D52" t="s">
         <v>25</v>
@@ -1849,10 +1852,10 @@
         <v>19</v>
       </c>
       <c r="B53" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C53" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D53" t="s">
         <v>25</v>
@@ -1872,10 +1875,10 @@
         <v>20</v>
       </c>
       <c r="B54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C54" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D54" t="s">
         <v>25</v>
@@ -1895,10 +1898,10 @@
         <v>21</v>
       </c>
       <c r="B55" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D55" t="s">
         <v>25</v>
@@ -1918,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="B56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C56" t="s">
         <v>26</v>
@@ -1941,7 +1944,7 @@
         <v>5</v>
       </c>
       <c r="B57" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C57" t="s">
         <v>26</v>
@@ -1964,7 +1967,7 @@
         <v>6</v>
       </c>
       <c r="B58" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C58" t="s">
         <v>26</v>
@@ -1987,7 +1990,7 @@
         <v>7</v>
       </c>
       <c r="B59" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C59" t="s">
         <v>26</v>
@@ -2010,7 +2013,7 @@
         <v>8</v>
       </c>
       <c r="B60" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C60" t="s">
         <v>26</v>
@@ -2033,7 +2036,7 @@
         <v>9</v>
       </c>
       <c r="B61" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C61" t="s">
         <v>26</v>
@@ -2056,7 +2059,7 @@
         <v>10</v>
       </c>
       <c r="B62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C62" t="s">
         <v>26</v>
@@ -2079,7 +2082,7 @@
         <v>11</v>
       </c>
       <c r="B63" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C63" t="s">
         <v>26</v>
@@ -2102,7 +2105,7 @@
         <v>12</v>
       </c>
       <c r="B64" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C64" t="s">
         <v>26</v>
@@ -2125,7 +2128,7 @@
         <v>13</v>
       </c>
       <c r="B65" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C65" t="s">
         <v>26</v>
@@ -2148,7 +2151,7 @@
         <v>14</v>
       </c>
       <c r="B66" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C66" t="s">
         <v>26</v>
@@ -2171,7 +2174,7 @@
         <v>15</v>
       </c>
       <c r="B67" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C67" t="s">
         <v>26</v>
@@ -2194,7 +2197,7 @@
         <v>16</v>
       </c>
       <c r="B68" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C68" t="s">
         <v>26</v>
@@ -2217,7 +2220,7 @@
         <v>17</v>
       </c>
       <c r="B69" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C69" t="s">
         <v>26</v>
@@ -2240,7 +2243,7 @@
         <v>18</v>
       </c>
       <c r="B70" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C70" t="s">
         <v>26</v>
@@ -2263,7 +2266,7 @@
         <v>19</v>
       </c>
       <c r="B71" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C71" t="s">
         <v>26</v>
@@ -2286,7 +2289,7 @@
         <v>20</v>
       </c>
       <c r="B72" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C72" t="s">
         <v>26</v>
@@ -2309,7 +2312,7 @@
         <v>21</v>
       </c>
       <c r="B73" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C73" t="s">
         <v>26</v>
@@ -2332,7 +2335,7 @@
         <v>4</v>
       </c>
       <c r="B74" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C74" t="s">
         <v>66</v>
@@ -2355,7 +2358,7 @@
         <v>5</v>
       </c>
       <c r="B75" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C75" t="s">
         <v>66</v>
@@ -2378,7 +2381,7 @@
         <v>6</v>
       </c>
       <c r="B76" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C76" t="s">
         <v>66</v>
@@ -2401,7 +2404,7 @@
         <v>7</v>
       </c>
       <c r="B77" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C77" t="s">
         <v>66</v>
@@ -2424,7 +2427,7 @@
         <v>8</v>
       </c>
       <c r="B78" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C78" t="s">
         <v>66</v>
@@ -2447,7 +2450,7 @@
         <v>9</v>
       </c>
       <c r="B79" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C79" t="s">
         <v>66</v>
@@ -2470,7 +2473,7 @@
         <v>10</v>
       </c>
       <c r="B80" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C80" t="s">
         <v>66</v>
@@ -2493,7 +2496,7 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C81" t="s">
         <v>66</v>
@@ -2516,7 +2519,7 @@
         <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C82" t="s">
         <v>66</v>
@@ -2539,7 +2542,7 @@
         <v>13</v>
       </c>
       <c r="B83" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C83" t="s">
         <v>66</v>
@@ -2562,7 +2565,7 @@
         <v>14</v>
       </c>
       <c r="B84" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C84" t="s">
         <v>66</v>
@@ -2585,7 +2588,7 @@
         <v>15</v>
       </c>
       <c r="B85" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C85" t="s">
         <v>66</v>
@@ -2608,7 +2611,7 @@
         <v>16</v>
       </c>
       <c r="B86" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C86" t="s">
         <v>66</v>
@@ -2631,7 +2634,7 @@
         <v>17</v>
       </c>
       <c r="B87" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C87" t="s">
         <v>66</v>
@@ -2654,7 +2657,7 @@
         <v>18</v>
       </c>
       <c r="B88" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C88" t="s">
         <v>66</v>
@@ -2677,7 +2680,7 @@
         <v>19</v>
       </c>
       <c r="B89" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C89" t="s">
         <v>66</v>
@@ -2700,7 +2703,7 @@
         <v>20</v>
       </c>
       <c r="B90" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C90" t="s">
         <v>66</v>
@@ -2723,7 +2726,7 @@
         <v>21</v>
       </c>
       <c r="B91" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C91" t="s">
         <v>66</v>
@@ -2746,7 +2749,7 @@
         <v>4</v>
       </c>
       <c r="B92" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C92" t="s">
         <v>66</v>
@@ -2769,7 +2772,7 @@
         <v>5</v>
       </c>
       <c r="B93" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C93" t="s">
         <v>66</v>
@@ -2792,7 +2795,7 @@
         <v>6</v>
       </c>
       <c r="B94" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C94" t="s">
         <v>66</v>
@@ -2815,7 +2818,7 @@
         <v>7</v>
       </c>
       <c r="B95" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C95" t="s">
         <v>66</v>
@@ -2838,7 +2841,7 @@
         <v>8</v>
       </c>
       <c r="B96" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C96" t="s">
         <v>66</v>
@@ -2861,7 +2864,7 @@
         <v>9</v>
       </c>
       <c r="B97" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C97" t="s">
         <v>66</v>
@@ -2884,7 +2887,7 @@
         <v>10</v>
       </c>
       <c r="B98" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C98" t="s">
         <v>66</v>
@@ -2907,7 +2910,7 @@
         <v>11</v>
       </c>
       <c r="B99" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C99" t="s">
         <v>66</v>
@@ -2930,7 +2933,7 @@
         <v>12</v>
       </c>
       <c r="B100" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C100" t="s">
         <v>66</v>
@@ -2953,7 +2956,7 @@
         <v>13</v>
       </c>
       <c r="B101" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C101" t="s">
         <v>66</v>
@@ -2976,7 +2979,7 @@
         <v>14</v>
       </c>
       <c r="B102" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C102" t="s">
         <v>66</v>
@@ -2999,7 +3002,7 @@
         <v>15</v>
       </c>
       <c r="B103" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C103" t="s">
         <v>66</v>
@@ -3022,7 +3025,7 @@
         <v>16</v>
       </c>
       <c r="B104" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C104" t="s">
         <v>66</v>
@@ -3045,7 +3048,7 @@
         <v>17</v>
       </c>
       <c r="B105" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C105" t="s">
         <v>66</v>
@@ -3068,7 +3071,7 @@
         <v>18</v>
       </c>
       <c r="B106" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C106" t="s">
         <v>66</v>
@@ -3091,7 +3094,7 @@
         <v>19</v>
       </c>
       <c r="B107" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C107" t="s">
         <v>66</v>
@@ -3114,7 +3117,7 @@
         <v>20</v>
       </c>
       <c r="B108" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C108" t="s">
         <v>66</v>
@@ -3137,7 +3140,7 @@
         <v>21</v>
       </c>
       <c r="B109" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C109" t="s">
         <v>66</v>
@@ -3160,10 +3163,10 @@
         <v>4</v>
       </c>
       <c r="B110" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C110" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D110" t="s">
         <v>30</v>
@@ -3183,10 +3186,10 @@
         <v>5</v>
       </c>
       <c r="B111" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C111" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D111" t="s">
         <v>30</v>
@@ -3206,10 +3209,10 @@
         <v>6</v>
       </c>
       <c r="B112" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C112" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D112" t="s">
         <v>30</v>
@@ -3229,10 +3232,10 @@
         <v>7</v>
       </c>
       <c r="B113" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C113" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D113" t="s">
         <v>30</v>
@@ -3252,10 +3255,10 @@
         <v>8</v>
       </c>
       <c r="B114" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C114" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D114" t="s">
         <v>30</v>
@@ -3275,10 +3278,10 @@
         <v>9</v>
       </c>
       <c r="B115" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C115" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D115" t="s">
         <v>30</v>
@@ -3298,10 +3301,10 @@
         <v>10</v>
       </c>
       <c r="B116" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C116" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D116" t="s">
         <v>30</v>
@@ -3321,10 +3324,10 @@
         <v>11</v>
       </c>
       <c r="B117" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C117" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D117" t="s">
         <v>30</v>
@@ -3344,10 +3347,10 @@
         <v>12</v>
       </c>
       <c r="B118" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C118" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D118" t="s">
         <v>30</v>
@@ -3367,10 +3370,10 @@
         <v>13</v>
       </c>
       <c r="B119" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C119" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D119" t="s">
         <v>30</v>
@@ -3390,10 +3393,10 @@
         <v>14</v>
       </c>
       <c r="B120" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C120" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D120" t="s">
         <v>30</v>
@@ -3413,10 +3416,10 @@
         <v>15</v>
       </c>
       <c r="B121" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C121" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D121" t="s">
         <v>30</v>
@@ -3436,10 +3439,10 @@
         <v>16</v>
       </c>
       <c r="B122" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C122" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D122" t="s">
         <v>30</v>
@@ -3459,10 +3462,10 @@
         <v>17</v>
       </c>
       <c r="B123" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C123" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D123" t="s">
         <v>30</v>
@@ -3482,10 +3485,10 @@
         <v>18</v>
       </c>
       <c r="B124" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C124" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D124" t="s">
         <v>30</v>
@@ -3505,10 +3508,10 @@
         <v>19</v>
       </c>
       <c r="B125" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C125" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D125" t="s">
         <v>30</v>
@@ -3528,10 +3531,10 @@
         <v>20</v>
       </c>
       <c r="B126" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C126" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D126" t="s">
         <v>30</v>
@@ -3551,10 +3554,10 @@
         <v>21</v>
       </c>
       <c r="B127" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C127" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D127" t="s">
         <v>30</v>
@@ -3574,7 +3577,7 @@
         <v>4</v>
       </c>
       <c r="B128" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C128" t="s">
         <v>66</v>
@@ -3597,7 +3600,7 @@
         <v>5</v>
       </c>
       <c r="B129" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C129" t="s">
         <v>66</v>
@@ -3620,7 +3623,7 @@
         <v>6</v>
       </c>
       <c r="B130" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C130" t="s">
         <v>66</v>
@@ -3643,7 +3646,7 @@
         <v>7</v>
       </c>
       <c r="B131" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C131" t="s">
         <v>66</v>
@@ -3666,7 +3669,7 @@
         <v>8</v>
       </c>
       <c r="B132" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C132" t="s">
         <v>66</v>
@@ -3689,7 +3692,7 @@
         <v>9</v>
       </c>
       <c r="B133" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C133" t="s">
         <v>66</v>
@@ -3712,7 +3715,7 @@
         <v>10</v>
       </c>
       <c r="B134" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C134" t="s">
         <v>66</v>
@@ -3735,7 +3738,7 @@
         <v>11</v>
       </c>
       <c r="B135" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C135" t="s">
         <v>66</v>
@@ -3758,7 +3761,7 @@
         <v>12</v>
       </c>
       <c r="B136" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C136" t="s">
         <v>66</v>
@@ -3781,7 +3784,7 @@
         <v>13</v>
       </c>
       <c r="B137" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C137" t="s">
         <v>66</v>
@@ -3804,7 +3807,7 @@
         <v>14</v>
       </c>
       <c r="B138" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C138" t="s">
         <v>66</v>
@@ -3827,7 +3830,7 @@
         <v>15</v>
       </c>
       <c r="B139" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C139" t="s">
         <v>66</v>
@@ -3850,7 +3853,7 @@
         <v>16</v>
       </c>
       <c r="B140" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C140" t="s">
         <v>66</v>
@@ -3873,7 +3876,7 @@
         <v>17</v>
       </c>
       <c r="B141" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C141" t="s">
         <v>66</v>
@@ -3896,7 +3899,7 @@
         <v>18</v>
       </c>
       <c r="B142" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C142" t="s">
         <v>66</v>
@@ -3919,7 +3922,7 @@
         <v>19</v>
       </c>
       <c r="B143" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C143" t="s">
         <v>66</v>
@@ -3942,7 +3945,7 @@
         <v>20</v>
       </c>
       <c r="B144" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C144" t="s">
         <v>66</v>
@@ -3965,7 +3968,7 @@
         <v>21</v>
       </c>
       <c r="B145" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C145" t="s">
         <v>66</v>
@@ -3988,7 +3991,7 @@
         <v>4</v>
       </c>
       <c r="B146" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C146" t="s">
         <v>35</v>
@@ -4011,7 +4014,7 @@
         <v>5</v>
       </c>
       <c r="B147" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C147" t="s">
         <v>35</v>
@@ -4034,7 +4037,7 @@
         <v>6</v>
       </c>
       <c r="B148" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C148" t="s">
         <v>35</v>
@@ -4057,7 +4060,7 @@
         <v>7</v>
       </c>
       <c r="B149" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C149" t="s">
         <v>35</v>
@@ -4080,7 +4083,7 @@
         <v>8</v>
       </c>
       <c r="B150" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C150" t="s">
         <v>35</v>
@@ -4103,7 +4106,7 @@
         <v>9</v>
       </c>
       <c r="B151" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C151" t="s">
         <v>35</v>
@@ -4126,7 +4129,7 @@
         <v>10</v>
       </c>
       <c r="B152" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C152" t="s">
         <v>35</v>
@@ -4149,7 +4152,7 @@
         <v>11</v>
       </c>
       <c r="B153" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C153" t="s">
         <v>35</v>
@@ -4172,7 +4175,7 @@
         <v>12</v>
       </c>
       <c r="B154" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C154" t="s">
         <v>35</v>
@@ -4195,7 +4198,7 @@
         <v>13</v>
       </c>
       <c r="B155" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C155" t="s">
         <v>35</v>
@@ -4218,7 +4221,7 @@
         <v>14</v>
       </c>
       <c r="B156" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C156" t="s">
         <v>35</v>
@@ -4241,7 +4244,7 @@
         <v>15</v>
       </c>
       <c r="B157" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C157" t="s">
         <v>35</v>
@@ -4264,7 +4267,7 @@
         <v>16</v>
       </c>
       <c r="B158" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C158" t="s">
         <v>35</v>
@@ -4287,7 +4290,7 @@
         <v>17</v>
       </c>
       <c r="B159" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C159" t="s">
         <v>35</v>
@@ -4310,7 +4313,7 @@
         <v>18</v>
       </c>
       <c r="B160" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C160" t="s">
         <v>35</v>
@@ -4333,7 +4336,7 @@
         <v>19</v>
       </c>
       <c r="B161" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C161" t="s">
         <v>35</v>
@@ -4356,7 +4359,7 @@
         <v>20</v>
       </c>
       <c r="B162" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C162" t="s">
         <v>35</v>
@@ -4379,7 +4382,7 @@
         <v>21</v>
       </c>
       <c r="B163" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C163" t="s">
         <v>35</v>
@@ -4402,7 +4405,7 @@
         <v>4</v>
       </c>
       <c r="B164" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C164" t="s">
         <v>35</v>
@@ -4425,7 +4428,7 @@
         <v>5</v>
       </c>
       <c r="B165" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C165" t="s">
         <v>35</v>
@@ -4448,7 +4451,7 @@
         <v>6</v>
       </c>
       <c r="B166" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C166" t="s">
         <v>35</v>
@@ -4471,7 +4474,7 @@
         <v>7</v>
       </c>
       <c r="B167" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C167" t="s">
         <v>35</v>
@@ -4494,7 +4497,7 @@
         <v>8</v>
       </c>
       <c r="B168" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C168" t="s">
         <v>35</v>
@@ -4517,7 +4520,7 @@
         <v>9</v>
       </c>
       <c r="B169" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C169" t="s">
         <v>35</v>
@@ -4540,7 +4543,7 @@
         <v>10</v>
       </c>
       <c r="B170" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C170" t="s">
         <v>35</v>
@@ -4563,7 +4566,7 @@
         <v>11</v>
       </c>
       <c r="B171" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C171" t="s">
         <v>35</v>
@@ -4586,7 +4589,7 @@
         <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C172" t="s">
         <v>35</v>
@@ -4609,7 +4612,7 @@
         <v>13</v>
       </c>
       <c r="B173" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C173" t="s">
         <v>35</v>
@@ -4632,7 +4635,7 @@
         <v>14</v>
       </c>
       <c r="B174" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C174" t="s">
         <v>35</v>
@@ -4655,7 +4658,7 @@
         <v>15</v>
       </c>
       <c r="B175" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C175" t="s">
         <v>35</v>
@@ -4678,7 +4681,7 @@
         <v>16</v>
       </c>
       <c r="B176" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C176" t="s">
         <v>35</v>
@@ -4701,7 +4704,7 @@
         <v>17</v>
       </c>
       <c r="B177" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C177" t="s">
         <v>35</v>
@@ -4724,7 +4727,7 @@
         <v>18</v>
       </c>
       <c r="B178" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C178" t="s">
         <v>35</v>
@@ -4747,7 +4750,7 @@
         <v>19</v>
       </c>
       <c r="B179" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C179" t="s">
         <v>35</v>
@@ -4770,7 +4773,7 @@
         <v>20</v>
       </c>
       <c r="B180" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C180" t="s">
         <v>35</v>
@@ -4793,7 +4796,7 @@
         <v>21</v>
       </c>
       <c r="B181" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C181" t="s">
         <v>35</v>
@@ -5647,7 +5650,7 @@
         <v>34</v>
       </c>
       <c r="C218" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D218" t="s">
         <v>40</v>
@@ -5670,7 +5673,7 @@
         <v>34</v>
       </c>
       <c r="C219" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D219" t="s">
         <v>40</v>
@@ -5693,7 +5696,7 @@
         <v>34</v>
       </c>
       <c r="C220" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D220" t="s">
         <v>40</v>
@@ -5716,7 +5719,7 @@
         <v>34</v>
       </c>
       <c r="C221" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D221" t="s">
         <v>40</v>
@@ -5739,7 +5742,7 @@
         <v>34</v>
       </c>
       <c r="C222" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D222" t="s">
         <v>40</v>
@@ -5762,7 +5765,7 @@
         <v>34</v>
       </c>
       <c r="C223" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D223" t="s">
         <v>40</v>
@@ -5785,7 +5788,7 @@
         <v>34</v>
       </c>
       <c r="C224" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D224" t="s">
         <v>40</v>
@@ -5808,7 +5811,7 @@
         <v>34</v>
       </c>
       <c r="C225" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D225" t="s">
         <v>40</v>
@@ -5831,7 +5834,7 @@
         <v>34</v>
       </c>
       <c r="C226" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D226" t="s">
         <v>40</v>
@@ -5854,7 +5857,7 @@
         <v>34</v>
       </c>
       <c r="C227" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D227" t="s">
         <v>40</v>
@@ -5877,7 +5880,7 @@
         <v>34</v>
       </c>
       <c r="C228" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D228" t="s">
         <v>40</v>
@@ -5900,7 +5903,7 @@
         <v>34</v>
       </c>
       <c r="C229" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D229" t="s">
         <v>40</v>
@@ -5923,7 +5926,7 @@
         <v>34</v>
       </c>
       <c r="C230" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D230" t="s">
         <v>40</v>
@@ -5946,7 +5949,7 @@
         <v>34</v>
       </c>
       <c r="C231" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D231" t="s">
         <v>40</v>
@@ -5969,7 +5972,7 @@
         <v>34</v>
       </c>
       <c r="C232" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D232" t="s">
         <v>40</v>
@@ -5992,7 +5995,7 @@
         <v>34</v>
       </c>
       <c r="C233" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D233" t="s">
         <v>40</v>
@@ -6015,7 +6018,7 @@
         <v>34</v>
       </c>
       <c r="C234" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D234" t="s">
         <v>40</v>
@@ -6038,7 +6041,7 @@
         <v>34</v>
       </c>
       <c r="C235" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D235" t="s">
         <v>40</v>
@@ -6475,7 +6478,7 @@
         <v>34</v>
       </c>
       <c r="C254" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D254" t="s">
         <v>42</v>
@@ -6498,7 +6501,7 @@
         <v>34</v>
       </c>
       <c r="C255" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D255" t="s">
         <v>42</v>
@@ -6521,7 +6524,7 @@
         <v>34</v>
       </c>
       <c r="C256" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D256" t="s">
         <v>42</v>
@@ -6544,7 +6547,7 @@
         <v>34</v>
       </c>
       <c r="C257" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D257" t="s">
         <v>42</v>
@@ -6567,7 +6570,7 @@
         <v>34</v>
       </c>
       <c r="C258" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D258" t="s">
         <v>42</v>
@@ -6590,7 +6593,7 @@
         <v>34</v>
       </c>
       <c r="C259" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D259" t="s">
         <v>42</v>
@@ -6613,7 +6616,7 @@
         <v>34</v>
       </c>
       <c r="C260" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D260" t="s">
         <v>42</v>
@@ -6636,7 +6639,7 @@
         <v>34</v>
       </c>
       <c r="C261" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D261" t="s">
         <v>42</v>
@@ -6659,7 +6662,7 @@
         <v>34</v>
       </c>
       <c r="C262" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D262" t="s">
         <v>42</v>
@@ -6682,7 +6685,7 @@
         <v>34</v>
       </c>
       <c r="C263" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D263" t="s">
         <v>42</v>
@@ -6705,7 +6708,7 @@
         <v>34</v>
       </c>
       <c r="C264" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D264" t="s">
         <v>42</v>
@@ -6728,7 +6731,7 @@
         <v>34</v>
       </c>
       <c r="C265" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D265" t="s">
         <v>42</v>
@@ -6751,7 +6754,7 @@
         <v>34</v>
       </c>
       <c r="C266" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D266" t="s">
         <v>42</v>
@@ -6774,7 +6777,7 @@
         <v>34</v>
       </c>
       <c r="C267" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D267" t="s">
         <v>42</v>
@@ -6797,7 +6800,7 @@
         <v>34</v>
       </c>
       <c r="C268" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D268" t="s">
         <v>42</v>
@@ -6820,7 +6823,7 @@
         <v>34</v>
       </c>
       <c r="C269" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D269" t="s">
         <v>42</v>
@@ -6843,7 +6846,7 @@
         <v>34</v>
       </c>
       <c r="C270" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D270" t="s">
         <v>42</v>
@@ -6866,7 +6869,7 @@
         <v>34</v>
       </c>
       <c r="C271" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D271" t="s">
         <v>42</v>
@@ -8131,7 +8134,7 @@
         <v>36</v>
       </c>
       <c r="C326" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D326" t="s">
         <v>46</v>
@@ -8154,7 +8157,7 @@
         <v>36</v>
       </c>
       <c r="C327" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D327" t="s">
         <v>46</v>
@@ -8177,7 +8180,7 @@
         <v>36</v>
       </c>
       <c r="C328" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D328" t="s">
         <v>46</v>
@@ -8200,7 +8203,7 @@
         <v>36</v>
       </c>
       <c r="C329" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D329" t="s">
         <v>46</v>
@@ -8223,7 +8226,7 @@
         <v>36</v>
       </c>
       <c r="C330" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D330" t="s">
         <v>46</v>
@@ -8246,7 +8249,7 @@
         <v>36</v>
       </c>
       <c r="C331" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D331" t="s">
         <v>46</v>
@@ -8269,7 +8272,7 @@
         <v>36</v>
       </c>
       <c r="C332" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D332" t="s">
         <v>46</v>
@@ -8292,7 +8295,7 @@
         <v>36</v>
       </c>
       <c r="C333" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D333" t="s">
         <v>46</v>
@@ -8315,7 +8318,7 @@
         <v>36</v>
       </c>
       <c r="C334" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D334" t="s">
         <v>46</v>
@@ -8338,7 +8341,7 @@
         <v>36</v>
       </c>
       <c r="C335" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D335" t="s">
         <v>46</v>
@@ -8361,7 +8364,7 @@
         <v>36</v>
       </c>
       <c r="C336" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D336" t="s">
         <v>46</v>
@@ -8384,7 +8387,7 @@
         <v>36</v>
       </c>
       <c r="C337" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D337" t="s">
         <v>46</v>
@@ -8407,7 +8410,7 @@
         <v>36</v>
       </c>
       <c r="C338" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D338" t="s">
         <v>46</v>
@@ -8430,7 +8433,7 @@
         <v>36</v>
       </c>
       <c r="C339" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D339" t="s">
         <v>46</v>
@@ -8453,7 +8456,7 @@
         <v>36</v>
       </c>
       <c r="C340" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D340" t="s">
         <v>46</v>
@@ -8476,7 +8479,7 @@
         <v>36</v>
       </c>
       <c r="C341" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D341" t="s">
         <v>46</v>
@@ -8499,7 +8502,7 @@
         <v>36</v>
       </c>
       <c r="C342" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D342" t="s">
         <v>46</v>
@@ -8522,7 +8525,7 @@
         <v>36</v>
       </c>
       <c r="C343" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D343" t="s">
         <v>46</v>
@@ -9787,10 +9790,10 @@
         <v>36</v>
       </c>
       <c r="C398" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D398" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E398">
         <v>2</v>
@@ -9810,10 +9813,10 @@
         <v>36</v>
       </c>
       <c r="C399" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D399" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E399">
         <v>2</v>
@@ -9833,10 +9836,10 @@
         <v>36</v>
       </c>
       <c r="C400" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D400" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E400">
         <v>2</v>
@@ -9856,10 +9859,10 @@
         <v>36</v>
       </c>
       <c r="C401" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D401" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E401">
         <v>4</v>
@@ -9879,10 +9882,10 @@
         <v>36</v>
       </c>
       <c r="C402" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D402" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E402">
         <v>2</v>
@@ -9902,10 +9905,10 @@
         <v>36</v>
       </c>
       <c r="C403" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D403" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E403">
         <v>2</v>
@@ -9925,10 +9928,10 @@
         <v>36</v>
       </c>
       <c r="C404" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D404" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E404">
         <v>2</v>
@@ -9948,10 +9951,10 @@
         <v>36</v>
       </c>
       <c r="C405" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D405" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E405">
         <v>2</v>
@@ -9971,10 +9974,10 @@
         <v>36</v>
       </c>
       <c r="C406" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D406" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E406">
         <v>4</v>
@@ -9994,10 +9997,10 @@
         <v>36</v>
       </c>
       <c r="C407" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D407" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E407">
         <v>2</v>
@@ -10017,10 +10020,10 @@
         <v>36</v>
       </c>
       <c r="C408" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D408" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E408" s="1">
         <v>2</v>
@@ -10040,10 +10043,10 @@
         <v>36</v>
       </c>
       <c r="C409" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D409" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E409">
         <v>4</v>
@@ -10063,10 +10066,10 @@
         <v>36</v>
       </c>
       <c r="C410" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D410" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E410">
         <v>2</v>
@@ -10086,10 +10089,10 @@
         <v>36</v>
       </c>
       <c r="C411" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D411" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E411">
         <v>4</v>
@@ -10109,10 +10112,10 @@
         <v>36</v>
       </c>
       <c r="C412" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D412" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E412">
         <v>4</v>
@@ -10132,10 +10135,10 @@
         <v>36</v>
       </c>
       <c r="C413" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D413" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E413">
         <v>2</v>
@@ -10155,10 +10158,10 @@
         <v>36</v>
       </c>
       <c r="C414" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D414" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E414">
         <v>4</v>
@@ -10178,10 +10181,10 @@
         <v>36</v>
       </c>
       <c r="C415" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="D415" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E415">
         <v>1</v>
@@ -10201,7 +10204,7 @@
         <v>36</v>
       </c>
       <c r="C416" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D416" t="s">
         <v>37</v>
@@ -10224,7 +10227,7 @@
         <v>36</v>
       </c>
       <c r="C417" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D417" t="s">
         <v>37</v>
@@ -10247,7 +10250,7 @@
         <v>36</v>
       </c>
       <c r="C418" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D418" t="s">
         <v>37</v>
@@ -10270,7 +10273,7 @@
         <v>36</v>
       </c>
       <c r="C419" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D419" t="s">
         <v>37</v>
@@ -10293,7 +10296,7 @@
         <v>36</v>
       </c>
       <c r="C420" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D420" t="s">
         <v>37</v>
@@ -10316,7 +10319,7 @@
         <v>36</v>
       </c>
       <c r="C421" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D421" t="s">
         <v>37</v>
@@ -10339,7 +10342,7 @@
         <v>36</v>
       </c>
       <c r="C422" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D422" t="s">
         <v>37</v>
@@ -10362,7 +10365,7 @@
         <v>36</v>
       </c>
       <c r="C423" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D423" t="s">
         <v>37</v>
@@ -10385,7 +10388,7 @@
         <v>36</v>
       </c>
       <c r="C424" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D424" t="s">
         <v>37</v>
@@ -10408,7 +10411,7 @@
         <v>36</v>
       </c>
       <c r="C425" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D425" t="s">
         <v>37</v>
@@ -10431,7 +10434,7 @@
         <v>36</v>
       </c>
       <c r="C426" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D426" t="s">
         <v>37</v>
@@ -10454,7 +10457,7 @@
         <v>36</v>
       </c>
       <c r="C427" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D427" t="s">
         <v>37</v>
@@ -10477,7 +10480,7 @@
         <v>36</v>
       </c>
       <c r="C428" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D428" t="s">
         <v>37</v>
@@ -10500,7 +10503,7 @@
         <v>36</v>
       </c>
       <c r="C429" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D429" t="s">
         <v>37</v>
@@ -10523,7 +10526,7 @@
         <v>36</v>
       </c>
       <c r="C430" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D430" t="s">
         <v>37</v>
@@ -10546,7 +10549,7 @@
         <v>36</v>
       </c>
       <c r="C431" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D431" t="s">
         <v>37</v>
@@ -10569,7 +10572,7 @@
         <v>36</v>
       </c>
       <c r="C432" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D432" t="s">
         <v>37</v>
@@ -10592,7 +10595,7 @@
         <v>36</v>
       </c>
       <c r="C433" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D433" t="s">
         <v>37</v>
@@ -11032,7 +11035,7 @@
         <v>35</v>
       </c>
       <c r="D452" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E452">
         <v>0</v>
@@ -11055,7 +11058,7 @@
         <v>35</v>
       </c>
       <c r="D453" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E453">
         <v>0</v>
@@ -11078,7 +11081,7 @@
         <v>35</v>
       </c>
       <c r="D454" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E454">
         <v>0</v>
@@ -11101,7 +11104,7 @@
         <v>35</v>
       </c>
       <c r="D455" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E455">
         <v>0</v>
@@ -11124,7 +11127,7 @@
         <v>35</v>
       </c>
       <c r="D456" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E456">
         <v>0</v>
@@ -11147,7 +11150,7 @@
         <v>35</v>
       </c>
       <c r="D457" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E457">
         <v>0</v>
@@ -11170,7 +11173,7 @@
         <v>35</v>
       </c>
       <c r="D458" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E458">
         <v>0</v>
@@ -11193,7 +11196,7 @@
         <v>35</v>
       </c>
       <c r="D459" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E459">
         <v>0</v>
@@ -11216,7 +11219,7 @@
         <v>35</v>
       </c>
       <c r="D460" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E460">
         <v>0</v>
@@ -11239,7 +11242,7 @@
         <v>35</v>
       </c>
       <c r="D461" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E461">
         <v>0</v>
@@ -11262,7 +11265,7 @@
         <v>35</v>
       </c>
       <c r="D462" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E462">
         <v>0</v>
@@ -11285,7 +11288,7 @@
         <v>35</v>
       </c>
       <c r="D463" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E463">
         <v>0</v>
@@ -11308,7 +11311,7 @@
         <v>35</v>
       </c>
       <c r="D464" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E464">
         <v>0</v>
@@ -11331,7 +11334,7 @@
         <v>35</v>
       </c>
       <c r="D465" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E465">
         <v>0</v>
@@ -11354,7 +11357,7 @@
         <v>35</v>
       </c>
       <c r="D466" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E466">
         <v>0</v>
@@ -11377,7 +11380,7 @@
         <v>35</v>
       </c>
       <c r="D467" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E467">
         <v>-1</v>
@@ -11400,7 +11403,7 @@
         <v>35</v>
       </c>
       <c r="D468" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E468">
         <v>0</v>
@@ -11423,7 +11426,7 @@
         <v>35</v>
       </c>
       <c r="D469" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E469">
         <v>0</v>

</xml_diff>